<commit_message>
Alignement entre LM FR et EHDS ec58a6db830b953e358c47fc661374e3cfca55b1
</commit_message>
<xml_diff>
--- a/modeleLogiqueEntete/ig/StructureDefinition-fr-encounter-care-document.xlsx
+++ b/modeleLogiqueEntete/ig/StructureDefinition-fr-encounter-care-document.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4358" uniqueCount="637">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4358" uniqueCount="636">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-09T09:28:52+00:00</t>
+    <t>2026-06-09T14:42:35+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1368,15 +1368,6 @@
   </si>
   <si>
     <t>Type de participation</t>
-  </si>
-  <si>
-    <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
-  &lt;coding&gt;
-    &lt;system value="https://mos.esante.gouv.fr/NOS/TRE_A13-HL7ParticipationType/FHIR/TRE-A13-HL7ParticipationType"/&gt;
-    &lt;code value="DIS"/&gt;
-    &lt;display value="Responsable de la sortie"/&gt;
-  &lt;/coding&gt;
-&lt;/valueCodeableConcept&gt;</t>
   </si>
   <si>
     <t>Encounter.participant:responsibleParty.period</t>
@@ -9957,7 +9948,7 @@
       </c>
       <c r="E68" s="2"/>
       <c r="F68" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G68" t="s" s="2">
         <v>79</v>
@@ -9992,7 +9983,7 @@
         <v>80</v>
       </c>
       <c r="S68" t="s" s="2">
-        <v>438</v>
+        <v>80</v>
       </c>
       <c r="T68" t="s" s="2">
         <v>80</v>
@@ -10060,7 +10051,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B69" t="s" s="2">
         <v>417</v>
@@ -10172,7 +10163,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B70" t="s" s="2">
         <v>422</v>
@@ -10198,10 +10189,10 @@
         <v>89</v>
       </c>
       <c r="K70" t="s" s="2">
+        <v>440</v>
+      </c>
+      <c r="L70" t="s" s="2">
         <v>441</v>
-      </c>
-      <c r="L70" t="s" s="2">
-        <v>442</v>
       </c>
       <c r="M70" t="s" s="2">
         <v>425</v>
@@ -10284,13 +10275,13 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B71" t="s" s="2">
         <v>399</v>
       </c>
       <c r="C71" t="s" s="2">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="D71" t="s" s="2">
         <v>80</v>
@@ -10315,7 +10306,7 @@
         <v>279</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="M71" t="s" s="2">
         <v>401</v>
@@ -10398,7 +10389,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B72" t="s" s="2">
         <v>406</v>
@@ -10510,7 +10501,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B73" t="s" s="2">
         <v>407</v>
@@ -10624,7 +10615,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B74" t="s" s="2">
         <v>408</v>
@@ -10740,7 +10731,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B75" t="s" s="2">
         <v>409</v>
@@ -10805,7 +10796,7 @@
       </c>
       <c r="Y75" s="2"/>
       <c r="Z75" t="s" s="2">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="AA75" t="s" s="2">
         <v>80</v>
@@ -10852,7 +10843,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B76" t="s" s="2">
         <v>417</v>
@@ -10964,7 +10955,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B77" t="s" s="2">
         <v>422</v>
@@ -10990,10 +10981,10 @@
         <v>89</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="L77" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="M77" t="s" s="2">
         <v>425</v>
@@ -11076,10 +11067,10 @@
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -11102,13 +11093,13 @@
         <v>89</v>
       </c>
       <c r="K78" t="s" s="2">
+        <v>454</v>
+      </c>
+      <c r="L78" t="s" s="2">
         <v>455</v>
       </c>
-      <c r="L78" t="s" s="2">
+      <c r="M78" t="s" s="2">
         <v>456</v>
-      </c>
-      <c r="M78" t="s" s="2">
-        <v>457</v>
       </c>
       <c r="N78" s="2"/>
       <c r="O78" s="2"/>
@@ -11159,7 +11150,7 @@
         <v>80</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>78</v>
@@ -11177,21 +11168,21 @@
         <v>397</v>
       </c>
       <c r="AL78" t="s" s="2">
+        <v>457</v>
+      </c>
+      <c r="AM78" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN78" t="s" s="2">
         <v>458</v>
-      </c>
-      <c r="AM78" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN78" t="s" s="2">
-        <v>459</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -11217,13 +11208,13 @@
         <v>254</v>
       </c>
       <c r="L79" t="s" s="2">
+        <v>460</v>
+      </c>
+      <c r="M79" t="s" s="2">
         <v>461</v>
       </c>
-      <c r="M79" t="s" s="2">
+      <c r="N79" t="s" s="2">
         <v>462</v>
-      </c>
-      <c r="N79" t="s" s="2">
-        <v>463</v>
       </c>
       <c r="O79" s="2"/>
       <c r="P79" t="s" s="2">
@@ -11273,7 +11264,7 @@
         <v>80</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>78</v>
@@ -11288,24 +11279,24 @@
         <v>100</v>
       </c>
       <c r="AK79" t="s" s="2">
+        <v>463</v>
+      </c>
+      <c r="AL79" t="s" s="2">
         <v>464</v>
       </c>
-      <c r="AL79" t="s" s="2">
+      <c r="AM79" t="s" s="2">
         <v>465</v>
       </c>
-      <c r="AM79" t="s" s="2">
+      <c r="AN79" t="s" s="2">
         <v>466</v>
-      </c>
-      <c r="AN79" t="s" s="2">
-        <v>467</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -11328,16 +11319,16 @@
         <v>80</v>
       </c>
       <c r="K80" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="L80" t="s" s="2">
         <v>469</v>
       </c>
-      <c r="L80" t="s" s="2">
+      <c r="M80" t="s" s="2">
         <v>470</v>
       </c>
-      <c r="M80" t="s" s="2">
+      <c r="N80" t="s" s="2">
         <v>471</v>
-      </c>
-      <c r="N80" t="s" s="2">
-        <v>472</v>
       </c>
       <c r="O80" s="2"/>
       <c r="P80" t="s" s="2">
@@ -11387,7 +11378,7 @@
         <v>80</v>
       </c>
       <c r="AF80" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="AG80" t="s" s="2">
         <v>78</v>
@@ -11402,28 +11393,28 @@
         <v>100</v>
       </c>
       <c r="AK80" t="s" s="2">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="AL80" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="AM80" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN80" t="s" s="2">
         <v>473</v>
-      </c>
-      <c r="AM80" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN80" t="s" s="2">
-        <v>474</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="E81" s="2"/>
       <c r="F81" t="s" s="2">
@@ -11445,13 +11436,13 @@
         <v>228</v>
       </c>
       <c r="L81" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="M81" t="s" s="2">
         <v>477</v>
       </c>
-      <c r="M81" t="s" s="2">
+      <c r="N81" t="s" s="2">
         <v>478</v>
-      </c>
-      <c r="N81" t="s" s="2">
-        <v>479</v>
       </c>
       <c r="O81" s="2"/>
       <c r="P81" t="s" s="2">
@@ -11480,11 +11471,11 @@
         <v>172</v>
       </c>
       <c r="Y81" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="Z81" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="Z81" t="s" s="2">
-        <v>481</v>
-      </c>
       <c r="AA81" t="s" s="2">
         <v>80</v>
       </c>
@@ -11501,7 +11492,7 @@
         <v>80</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>78</v>
@@ -11516,28 +11507,28 @@
         <v>100</v>
       </c>
       <c r="AK81" t="s" s="2">
+        <v>481</v>
+      </c>
+      <c r="AL81" t="s" s="2">
         <v>482</v>
       </c>
-      <c r="AL81" t="s" s="2">
+      <c r="AM81" t="s" s="2">
         <v>483</v>
       </c>
-      <c r="AM81" t="s" s="2">
+      <c r="AN81" t="s" s="2">
         <v>484</v>
-      </c>
-      <c r="AN81" t="s" s="2">
-        <v>485</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="E82" s="2"/>
       <c r="F82" t="s" s="2">
@@ -11556,16 +11547,16 @@
         <v>89</v>
       </c>
       <c r="K82" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="L82" t="s" s="2">
         <v>487</v>
       </c>
-      <c r="L82" t="s" s="2">
-        <v>488</v>
-      </c>
       <c r="M82" t="s" s="2">
+        <v>477</v>
+      </c>
+      <c r="N82" t="s" s="2">
         <v>478</v>
-      </c>
-      <c r="N82" t="s" s="2">
-        <v>479</v>
       </c>
       <c r="O82" s="2"/>
       <c r="P82" t="s" s="2">
@@ -11615,7 +11606,7 @@
         <v>80</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>78</v>
@@ -11630,24 +11621,24 @@
         <v>100</v>
       </c>
       <c r="AK82" t="s" s="2">
+        <v>481</v>
+      </c>
+      <c r="AL82" t="s" s="2">
         <v>482</v>
       </c>
-      <c r="AL82" t="s" s="2">
+      <c r="AM82" t="s" s="2">
         <v>483</v>
       </c>
-      <c r="AM82" t="s" s="2">
+      <c r="AN82" t="s" s="2">
         <v>484</v>
-      </c>
-      <c r="AN82" t="s" s="2">
-        <v>485</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="2">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -11673,10 +11664,10 @@
         <v>279</v>
       </c>
       <c r="L83" t="s" s="2">
+        <v>489</v>
+      </c>
+      <c r="M83" t="s" s="2">
         <v>490</v>
-      </c>
-      <c r="M83" t="s" s="2">
-        <v>491</v>
       </c>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
@@ -11727,7 +11718,7 @@
         <v>80</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>78</v>
@@ -11745,7 +11736,7 @@
         <v>80</v>
       </c>
       <c r="AL83" t="s" s="2">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="AM83" t="s" s="2">
         <v>80</v>
@@ -11756,10 +11747,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -11868,10 +11859,10 @@
     </row>
     <row r="85">
       <c r="A85" t="s" s="2">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -11982,10 +11973,10 @@
     </row>
     <row r="86">
       <c r="A86" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -12098,14 +12089,14 @@
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E87" s="2"/>
       <c r="F87" t="s" s="2">
@@ -12124,16 +12115,16 @@
         <v>89</v>
       </c>
       <c r="K87" t="s" s="2">
+        <v>497</v>
+      </c>
+      <c r="L87" t="s" s="2">
         <v>498</v>
       </c>
-      <c r="L87" t="s" s="2">
+      <c r="M87" t="s" s="2">
         <v>499</v>
       </c>
-      <c r="M87" t="s" s="2">
-        <v>500</v>
-      </c>
       <c r="N87" t="s" s="2">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="O87" s="2"/>
       <c r="P87" t="s" s="2">
@@ -12183,7 +12174,7 @@
         <v>80</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>88</v>
@@ -12198,24 +12189,24 @@
         <v>100</v>
       </c>
       <c r="AK87" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="AL87" t="s" s="2">
         <v>501</v>
       </c>
-      <c r="AL87" t="s" s="2">
+      <c r="AM87" t="s" s="2">
+        <v>483</v>
+      </c>
+      <c r="AN87" t="s" s="2">
         <v>502</v>
-      </c>
-      <c r="AM87" t="s" s="2">
-        <v>484</v>
-      </c>
-      <c r="AN87" t="s" s="2">
-        <v>503</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -12241,10 +12232,10 @@
         <v>228</v>
       </c>
       <c r="L88" t="s" s="2">
+        <v>504</v>
+      </c>
+      <c r="M88" t="s" s="2">
         <v>505</v>
-      </c>
-      <c r="M88" t="s" s="2">
-        <v>506</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -12274,11 +12265,11 @@
         <v>172</v>
       </c>
       <c r="Y88" t="s" s="2">
+        <v>506</v>
+      </c>
+      <c r="Z88" t="s" s="2">
         <v>507</v>
       </c>
-      <c r="Z88" t="s" s="2">
-        <v>508</v>
-      </c>
       <c r="AA88" t="s" s="2">
         <v>80</v>
       </c>
@@ -12295,7 +12286,7 @@
         <v>80</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>78</v>
@@ -12324,10 +12315,10 @@
     </row>
     <row r="89">
       <c r="A89" t="s" s="2">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -12350,13 +12341,13 @@
         <v>80</v>
       </c>
       <c r="K89" t="s" s="2">
+        <v>509</v>
+      </c>
+      <c r="L89" t="s" s="2">
         <v>510</v>
       </c>
-      <c r="L89" t="s" s="2">
+      <c r="M89" t="s" s="2">
         <v>511</v>
-      </c>
-      <c r="M89" t="s" s="2">
-        <v>512</v>
       </c>
       <c r="N89" s="2"/>
       <c r="O89" s="2"/>
@@ -12407,7 +12398,7 @@
         <v>80</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>78</v>
@@ -12425,7 +12416,7 @@
         <v>80</v>
       </c>
       <c r="AL89" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AM89" t="s" s="2">
         <v>80</v>
@@ -12436,10 +12427,10 @@
     </row>
     <row r="90">
       <c r="A90" t="s" s="2">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -12462,16 +12453,16 @@
         <v>80</v>
       </c>
       <c r="K90" t="s" s="2">
+        <v>514</v>
+      </c>
+      <c r="L90" t="s" s="2">
         <v>515</v>
       </c>
-      <c r="L90" t="s" s="2">
+      <c r="M90" t="s" s="2">
         <v>516</v>
       </c>
-      <c r="M90" t="s" s="2">
+      <c r="N90" t="s" s="2">
         <v>517</v>
-      </c>
-      <c r="N90" t="s" s="2">
-        <v>518</v>
       </c>
       <c r="O90" s="2"/>
       <c r="P90" t="s" s="2">
@@ -12521,7 +12512,7 @@
         <v>80</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>78</v>
@@ -12539,7 +12530,7 @@
         <v>80</v>
       </c>
       <c r="AL90" t="s" s="2">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="AM90" t="s" s="2">
         <v>80</v>
@@ -12550,10 +12541,10 @@
     </row>
     <row r="91">
       <c r="A91" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -12579,13 +12570,13 @@
         <v>279</v>
       </c>
       <c r="L91" t="s" s="2">
+        <v>520</v>
+      </c>
+      <c r="M91" t="s" s="2">
         <v>521</v>
       </c>
-      <c r="M91" t="s" s="2">
+      <c r="N91" t="s" s="2">
         <v>522</v>
-      </c>
-      <c r="N91" t="s" s="2">
-        <v>523</v>
       </c>
       <c r="O91" s="2"/>
       <c r="P91" t="s" s="2">
@@ -12635,7 +12626,7 @@
         <v>80</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>78</v>
@@ -12653,7 +12644,7 @@
         <v>80</v>
       </c>
       <c r="AL91" t="s" s="2">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AM91" t="s" s="2">
         <v>80</v>
@@ -12664,10 +12655,10 @@
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -12776,10 +12767,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -12890,10 +12881,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s" s="2">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -13006,10 +12997,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -13035,10 +13026,10 @@
         <v>208</v>
       </c>
       <c r="L95" t="s" s="2">
+        <v>528</v>
+      </c>
+      <c r="M95" t="s" s="2">
         <v>529</v>
-      </c>
-      <c r="M95" t="s" s="2">
-        <v>530</v>
       </c>
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
@@ -13089,7 +13080,7 @@
         <v>80</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>78</v>
@@ -13113,15 +13104,15 @@
         <v>80</v>
       </c>
       <c r="AN95" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -13230,10 +13221,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -13344,10 +13335,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -13460,10 +13451,10 @@
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -13492,7 +13483,7 @@
         <v>229</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="N99" t="s" s="2">
         <v>231</v>
@@ -13574,10 +13565,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -13606,7 +13597,7 @@
         <v>237</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="N100" t="s" s="2">
         <v>239</v>
@@ -13619,7 +13610,7 @@
       </c>
       <c r="Q100" s="2"/>
       <c r="R100" t="s" s="2">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="S100" t="s" s="2">
         <v>80</v>
@@ -13690,10 +13681,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -13804,10 +13795,10 @@
     </row>
     <row r="102">
       <c r="A102" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -13916,10 +13907,10 @@
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -14030,10 +14021,10 @@
     </row>
     <row r="104">
       <c r="A104" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -14056,13 +14047,13 @@
         <v>80</v>
       </c>
       <c r="K104" t="s" s="2">
+        <v>543</v>
+      </c>
+      <c r="L104" t="s" s="2">
         <v>544</v>
       </c>
-      <c r="L104" t="s" s="2">
+      <c r="M104" t="s" s="2">
         <v>545</v>
-      </c>
-      <c r="M104" t="s" s="2">
-        <v>546</v>
       </c>
       <c r="N104" s="2"/>
       <c r="O104" s="2"/>
@@ -14113,7 +14104,7 @@
         <v>80</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>78</v>
@@ -14131,7 +14122,7 @@
         <v>80</v>
       </c>
       <c r="AL104" t="s" s="2">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="AM104" t="s" s="2">
         <v>80</v>
@@ -14142,10 +14133,10 @@
     </row>
     <row r="105">
       <c r="A105" t="s" s="2">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -14171,10 +14162,10 @@
         <v>228</v>
       </c>
       <c r="L105" t="s" s="2">
+        <v>548</v>
+      </c>
+      <c r="M105" t="s" s="2">
         <v>549</v>
-      </c>
-      <c r="M105" t="s" s="2">
-        <v>550</v>
       </c>
       <c r="N105" s="2"/>
       <c r="O105" s="2"/>
@@ -14204,11 +14195,11 @@
         <v>172</v>
       </c>
       <c r="Y105" t="s" s="2">
+        <v>550</v>
+      </c>
+      <c r="Z105" t="s" s="2">
         <v>551</v>
       </c>
-      <c r="Z105" t="s" s="2">
-        <v>552</v>
-      </c>
       <c r="AA105" t="s" s="2">
         <v>80</v>
       </c>
@@ -14225,7 +14216,7 @@
         <v>80</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>78</v>
@@ -14243,21 +14234,21 @@
         <v>80</v>
       </c>
       <c r="AL105" t="s" s="2">
+        <v>552</v>
+      </c>
+      <c r="AM105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN105" t="s" s="2">
         <v>553</v>
-      </c>
-      <c r="AM105" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN105" t="s" s="2">
-        <v>554</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="s" s="2">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -14283,10 +14274,10 @@
         <v>228</v>
       </c>
       <c r="L106" t="s" s="2">
+        <v>555</v>
+      </c>
+      <c r="M106" t="s" s="2">
         <v>556</v>
-      </c>
-      <c r="M106" t="s" s="2">
-        <v>557</v>
       </c>
       <c r="N106" s="2"/>
       <c r="O106" s="2"/>
@@ -14316,11 +14307,11 @@
         <v>158</v>
       </c>
       <c r="Y106" t="s" s="2">
+        <v>557</v>
+      </c>
+      <c r="Z106" t="s" s="2">
         <v>558</v>
       </c>
-      <c r="Z106" t="s" s="2">
-        <v>559</v>
-      </c>
       <c r="AA106" t="s" s="2">
         <v>80</v>
       </c>
@@ -14337,7 +14328,7 @@
         <v>80</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>78</v>
@@ -14361,15 +14352,15 @@
         <v>80</v>
       </c>
       <c r="AN106" t="s" s="2">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -14395,16 +14386,16 @@
         <v>228</v>
       </c>
       <c r="L107" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="M107" t="s" s="2">
         <v>562</v>
       </c>
-      <c r="M107" t="s" s="2">
+      <c r="N107" t="s" s="2">
         <v>563</v>
       </c>
-      <c r="N107" t="s" s="2">
+      <c r="O107" t="s" s="2">
         <v>564</v>
-      </c>
-      <c r="O107" t="s" s="2">
-        <v>565</v>
       </c>
       <c r="P107" t="s" s="2">
         <v>80</v>
@@ -14432,11 +14423,11 @@
         <v>158</v>
       </c>
       <c r="Y107" t="s" s="2">
+        <v>565</v>
+      </c>
+      <c r="Z107" t="s" s="2">
         <v>566</v>
       </c>
-      <c r="Z107" t="s" s="2">
-        <v>567</v>
-      </c>
       <c r="AA107" t="s" s="2">
         <v>80</v>
       </c>
@@ -14453,7 +14444,7 @@
         <v>80</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>78</v>
@@ -14471,21 +14462,21 @@
         <v>80</v>
       </c>
       <c r="AL107" t="s" s="2">
+        <v>567</v>
+      </c>
+      <c r="AM107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN107" t="s" s="2">
         <v>568</v>
-      </c>
-      <c r="AM107" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN107" t="s" s="2">
-        <v>569</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s" s="2">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -14511,10 +14502,10 @@
         <v>228</v>
       </c>
       <c r="L108" t="s" s="2">
+        <v>570</v>
+      </c>
+      <c r="M108" t="s" s="2">
         <v>571</v>
-      </c>
-      <c r="M108" t="s" s="2">
-        <v>572</v>
       </c>
       <c r="N108" s="2"/>
       <c r="O108" s="2"/>
@@ -14544,11 +14535,11 @@
         <v>172</v>
       </c>
       <c r="Y108" t="s" s="2">
+        <v>572</v>
+      </c>
+      <c r="Z108" t="s" s="2">
         <v>573</v>
       </c>
-      <c r="Z108" t="s" s="2">
-        <v>574</v>
-      </c>
       <c r="AA108" t="s" s="2">
         <v>80</v>
       </c>
@@ -14565,7 +14556,7 @@
         <v>80</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>78</v>
@@ -14583,21 +14574,21 @@
         <v>80</v>
       </c>
       <c r="AL108" t="s" s="2">
+        <v>574</v>
+      </c>
+      <c r="AM108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN108" t="s" s="2">
         <v>575</v>
-      </c>
-      <c r="AM108" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN108" t="s" s="2">
-        <v>576</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -14623,10 +14614,10 @@
         <v>228</v>
       </c>
       <c r="L109" t="s" s="2">
+        <v>577</v>
+      </c>
+      <c r="M109" t="s" s="2">
         <v>578</v>
-      </c>
-      <c r="M109" t="s" s="2">
-        <v>579</v>
       </c>
       <c r="N109" s="2"/>
       <c r="O109" s="2"/>
@@ -14656,11 +14647,11 @@
         <v>172</v>
       </c>
       <c r="Y109" t="s" s="2">
+        <v>579</v>
+      </c>
+      <c r="Z109" t="s" s="2">
         <v>580</v>
       </c>
-      <c r="Z109" t="s" s="2">
-        <v>581</v>
-      </c>
       <c r="AA109" t="s" s="2">
         <v>80</v>
       </c>
@@ -14677,7 +14668,7 @@
         <v>80</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>78</v>
@@ -14695,21 +14686,21 @@
         <v>80</v>
       </c>
       <c r="AL109" t="s" s="2">
+        <v>581</v>
+      </c>
+      <c r="AM109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN109" t="s" s="2">
         <v>582</v>
-      </c>
-      <c r="AM109" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN109" t="s" s="2">
-        <v>583</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s" s="2">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -14732,13 +14723,13 @@
         <v>80</v>
       </c>
       <c r="K110" t="s" s="2">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="L110" t="s" s="2">
+        <v>584</v>
+      </c>
+      <c r="M110" t="s" s="2">
         <v>585</v>
-      </c>
-      <c r="M110" t="s" s="2">
-        <v>586</v>
       </c>
       <c r="N110" s="2"/>
       <c r="O110" s="2"/>
@@ -14789,7 +14780,7 @@
         <v>80</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>78</v>
@@ -14807,21 +14798,21 @@
         <v>80</v>
       </c>
       <c r="AL110" t="s" s="2">
+        <v>586</v>
+      </c>
+      <c r="AM110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN110" t="s" s="2">
         <v>587</v>
-      </c>
-      <c r="AM110" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN110" t="s" s="2">
-        <v>588</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -14847,10 +14838,10 @@
         <v>228</v>
       </c>
       <c r="L111" t="s" s="2">
+        <v>589</v>
+      </c>
+      <c r="M111" t="s" s="2">
         <v>590</v>
-      </c>
-      <c r="M111" t="s" s="2">
-        <v>591</v>
       </c>
       <c r="N111" s="2"/>
       <c r="O111" s="2"/>
@@ -14881,7 +14872,7 @@
       </c>
       <c r="Y111" s="2"/>
       <c r="Z111" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="AA111" t="s" s="2">
         <v>80</v>
@@ -14899,7 +14890,7 @@
         <v>80</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>78</v>
@@ -14917,21 +14908,21 @@
         <v>80</v>
       </c>
       <c r="AL111" t="s" s="2">
+        <v>592</v>
+      </c>
+      <c r="AM111" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN111" t="s" s="2">
         <v>593</v>
-      </c>
-      <c r="AM111" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN111" t="s" s="2">
-        <v>594</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -14957,13 +14948,13 @@
         <v>279</v>
       </c>
       <c r="L112" t="s" s="2">
+        <v>595</v>
+      </c>
+      <c r="M112" t="s" s="2">
         <v>596</v>
       </c>
-      <c r="M112" t="s" s="2">
+      <c r="N112" t="s" s="2">
         <v>597</v>
-      </c>
-      <c r="N112" t="s" s="2">
-        <v>598</v>
       </c>
       <c r="O112" s="2"/>
       <c r="P112" t="s" s="2">
@@ -15013,7 +15004,7 @@
         <v>80</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>78</v>
@@ -15031,7 +15022,7 @@
         <v>80</v>
       </c>
       <c r="AL112" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="AM112" t="s" s="2">
         <v>80</v>
@@ -15042,10 +15033,10 @@
     </row>
     <row r="113">
       <c r="A113" t="s" s="2">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -15154,10 +15145,10 @@
     </row>
     <row r="114">
       <c r="A114" t="s" s="2">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -15268,10 +15259,10 @@
     </row>
     <row r="115">
       <c r="A115" t="s" s="2">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
@@ -15384,10 +15375,10 @@
     </row>
     <row r="116">
       <c r="A116" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -15410,13 +15401,13 @@
         <v>80</v>
       </c>
       <c r="K116" t="s" s="2">
+        <v>603</v>
+      </c>
+      <c r="L116" t="s" s="2">
         <v>604</v>
       </c>
-      <c r="L116" t="s" s="2">
+      <c r="M116" t="s" s="2">
         <v>605</v>
-      </c>
-      <c r="M116" t="s" s="2">
-        <v>606</v>
       </c>
       <c r="N116" s="2"/>
       <c r="O116" s="2"/>
@@ -15467,7 +15458,7 @@
         <v>80</v>
       </c>
       <c r="AF116" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="AG116" t="s" s="2">
         <v>88</v>
@@ -15482,24 +15473,24 @@
         <v>100</v>
       </c>
       <c r="AK116" t="s" s="2">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="AL116" t="s" s="2">
         <v>427</v>
       </c>
       <c r="AM116" t="s" s="2">
+        <v>607</v>
+      </c>
+      <c r="AN116" t="s" s="2">
         <v>608</v>
-      </c>
-      <c r="AN116" t="s" s="2">
-        <v>609</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -15525,13 +15516,13 @@
         <v>168</v>
       </c>
       <c r="L117" t="s" s="2">
+        <v>610</v>
+      </c>
+      <c r="M117" t="s" s="2">
         <v>611</v>
       </c>
-      <c r="M117" t="s" s="2">
+      <c r="N117" t="s" s="2">
         <v>612</v>
-      </c>
-      <c r="N117" t="s" s="2">
-        <v>613</v>
       </c>
       <c r="O117" s="2"/>
       <c r="P117" t="s" s="2">
@@ -15560,11 +15551,11 @@
         <v>222</v>
       </c>
       <c r="Y117" t="s" s="2">
+        <v>613</v>
+      </c>
+      <c r="Z117" t="s" s="2">
         <v>614</v>
       </c>
-      <c r="Z117" t="s" s="2">
-        <v>615</v>
-      </c>
       <c r="AA117" t="s" s="2">
         <v>80</v>
       </c>
@@ -15581,7 +15572,7 @@
         <v>80</v>
       </c>
       <c r="AF117" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="AG117" t="s" s="2">
         <v>78</v>
@@ -15599,7 +15590,7 @@
         <v>80</v>
       </c>
       <c r="AL117" t="s" s="2">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="AM117" t="s" s="2">
         <v>80</v>
@@ -15610,10 +15601,10 @@
     </row>
     <row r="118">
       <c r="A118" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
@@ -15639,13 +15630,13 @@
         <v>228</v>
       </c>
       <c r="L118" t="s" s="2">
+        <v>617</v>
+      </c>
+      <c r="M118" t="s" s="2">
         <v>618</v>
       </c>
-      <c r="M118" t="s" s="2">
+      <c r="N118" t="s" s="2">
         <v>619</v>
-      </c>
-      <c r="N118" t="s" s="2">
-        <v>620</v>
       </c>
       <c r="O118" s="2"/>
       <c r="P118" t="s" s="2">
@@ -15675,7 +15666,7 @@
       </c>
       <c r="Y118" s="2"/>
       <c r="Z118" t="s" s="2">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="AA118" t="s" s="2">
         <v>80</v>
@@ -15693,7 +15684,7 @@
         <v>80</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>78</v>
@@ -15722,10 +15713,10 @@
     </row>
     <row r="119">
       <c r="A119" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" t="s" s="2">
@@ -15751,10 +15742,10 @@
         <v>254</v>
       </c>
       <c r="L119" t="s" s="2">
+        <v>622</v>
+      </c>
+      <c r="M119" t="s" s="2">
         <v>623</v>
-      </c>
-      <c r="M119" t="s" s="2">
-        <v>624</v>
       </c>
       <c r="N119" s="2"/>
       <c r="O119" s="2"/>
@@ -15805,7 +15796,7 @@
         <v>80</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>78</v>
@@ -15834,10 +15825,10 @@
     </row>
     <row r="120">
       <c r="A120" t="s" s="2">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -15863,10 +15854,10 @@
         <v>261</v>
       </c>
       <c r="L120" t="s" s="2">
+        <v>625</v>
+      </c>
+      <c r="M120" t="s" s="2">
         <v>626</v>
-      </c>
-      <c r="M120" t="s" s="2">
-        <v>627</v>
       </c>
       <c r="N120" s="2"/>
       <c r="O120" s="2"/>
@@ -15917,7 +15908,7 @@
         <v>80</v>
       </c>
       <c r="AF120" t="s" s="2">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="AG120" t="s" s="2">
         <v>78</v>
@@ -15935,21 +15926,21 @@
         <v>426</v>
       </c>
       <c r="AL120" t="s" s="2">
+        <v>627</v>
+      </c>
+      <c r="AM120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN120" t="s" s="2">
         <v>628</v>
-      </c>
-      <c r="AM120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN120" t="s" s="2">
-        <v>629</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s" s="2">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -15972,16 +15963,16 @@
         <v>80</v>
       </c>
       <c r="K121" t="s" s="2">
+        <v>630</v>
+      </c>
+      <c r="L121" t="s" s="2">
         <v>631</v>
       </c>
-      <c r="L121" t="s" s="2">
+      <c r="M121" t="s" s="2">
         <v>632</v>
       </c>
-      <c r="M121" t="s" s="2">
+      <c r="N121" t="s" s="2">
         <v>633</v>
-      </c>
-      <c r="N121" t="s" s="2">
-        <v>634</v>
       </c>
       <c r="O121" s="2"/>
       <c r="P121" t="s" s="2">
@@ -16031,7 +16022,7 @@
         <v>80</v>
       </c>
       <c r="AF121" t="s" s="2">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="AG121" t="s" s="2">
         <v>78</v>
@@ -16046,10 +16037,10 @@
         <v>100</v>
       </c>
       <c r="AK121" t="s" s="2">
+        <v>634</v>
+      </c>
+      <c r="AL121" t="s" s="2">
         <v>635</v>
-      </c>
-      <c r="AL121" t="s" s="2">
-        <v>636</v>
       </c>
       <c r="AM121" t="s" s="2">
         <v>80</v>

</xml_diff>